<commit_message>
feat: support group identifiers and subject assignments
</commit_message>
<xml_diff>
--- a/app/static/example.xlsx
+++ b/app/static/example.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\imluza\Downloads\Telegram Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\imuratov\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46F2629B-FC50-468F-8EE3-8E5CB9E44A72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="13890"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Дата</t>
   </si>
@@ -215,12 +214,18 @@
       </rPr>
       <t xml:space="preserve">                         (не обязателен) </t>
     </r>
+  </si>
+  <si>
+    <t>Тема занятия</t>
+  </si>
+  <si>
+    <t>Например: Квадратные уравнения (не обязательно)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -680,21 +685,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" style="5" customWidth="1"/>
-    <col min="2" max="2" width="34.109375" style="6" customWidth="1"/>
-    <col min="3" max="3" width="26.21875" style="6" customWidth="1"/>
-    <col min="4" max="4" width="34.21875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="18.44140625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="23.109375" style="5" customWidth="1"/>
-    <col min="7" max="7" width="20.21875" style="5" customWidth="1"/>
-    <col min="8" max="8" width="16.77734375" style="5" customWidth="1"/>
+    <col min="1" max="1" width="24.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="34.140625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="26.28515625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="34.28515625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="23.140625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="20.28515625" style="5" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -719,8 +725,11 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" ht="83.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>8</v>
       </c>
@@ -744,6 +753,9 @@
       </c>
       <c r="H2" s="11" t="s">
         <v>15</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>